<commit_message>
Update ML multiclass model comparison results with correct 15-column leakage metrics
</commit_message>
<xml_diff>
--- a/dataset/15 Columns Leakage/ML_Multiclass_Model_Comparison_Results.xlsx
+++ b/dataset/15 Columns Leakage/ML_Multiclass_Model_Comparison_Results.xlsx
@@ -566,7 +566,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H65"/>
+  <dimension ref="A1:H70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -655,10 +655,10 @@
         </is>
       </c>
       <c r="G4" s="6" t="n">
-        <v>0.8881</v>
+        <v>0.8868</v>
       </c>
       <c r="H4" s="6" t="n">
-        <v>0.8862</v>
+        <v>0.8981</v>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
@@ -687,10 +687,10 @@
         </is>
       </c>
       <c r="G5" s="10" t="n">
-        <v>0.9475</v>
+        <v>0.9509</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>0.9454</v>
+        <v>0.9534</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
@@ -719,10 +719,10 @@
         </is>
       </c>
       <c r="G6" s="6" t="n">
-        <v>0.5963000000000001</v>
+        <v>0.5989</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>0.1245</v>
+        <v>0.1624</v>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
@@ -751,10 +751,10 @@
         </is>
       </c>
       <c r="G7" s="10" t="n">
-        <v>0.8739</v>
+        <v>0.8758</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>0.7069</v>
+        <v>0.7088</v>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
@@ -786,7 +786,7 @@
         <v>0.9426</v>
       </c>
       <c r="H8" s="6" t="n">
-        <v>0.7607</v>
+        <v>0.7674</v>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
@@ -815,439 +815,595 @@
         </is>
       </c>
       <c r="G9" s="10" t="n">
-        <v>0.6123</v>
+        <v>0.6179</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>0.1276</v>
-      </c>
-    </row>
-    <row r="10" ht="15" customHeight="1"/>
+        <v>0.151</v>
+      </c>
+    </row>
+    <row r="10" ht="15" customHeight="1">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>Diabetes All Drugs (10)</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="n">
+        <v>5208</v>
+      </c>
+      <c r="C10" s="8" t="n">
+        <v>2169</v>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>41.65%</t>
+        </is>
+      </c>
+      <c r="E10" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>Random Forest</t>
+        </is>
+      </c>
+      <c r="G10" s="10" t="n">
+        <v>0.8858</v>
+      </c>
+      <c r="H10" s="10" t="n">
+        <v>0.6942</v>
+      </c>
+    </row>
     <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="11" t="inlineStr">
-        <is>
-          <t>Imputation &amp; Preprocessing Methodology for outc_cod</t>
-        </is>
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Diabetes All Drugs (10)</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="n">
+        <v>5208</v>
+      </c>
+      <c r="C11" s="4" t="n">
+        <v>2169</v>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>41.65%</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="n">
+        <v>0.9357</v>
+      </c>
+      <c r="H11" s="6" t="n">
+        <v>0.736</v>
       </c>
     </row>
     <row r="12" ht="18" customHeight="1">
-      <c r="A12" s="12" t="inlineStr">
-        <is>
-          <t>The empty outcome values (5,933 in Obesity All, and 5,682 in Obesity Selected 4) were solved using a two-stage clinical imputation pipeline instead of simple deletion or filling with 'NS':</t>
-        </is>
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>Diabetes All Drugs (10)</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="n">
+        <v>5208</v>
+      </c>
+      <c r="C12" s="8" t="n">
+        <v>2169</v>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>41.65%</t>
+        </is>
+      </c>
+      <c r="E12" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>HANConv GNN</t>
+        </is>
+      </c>
+      <c r="G12" s="10" t="n">
+        <v>0.5518</v>
+      </c>
+      <c r="H12" s="10" t="n">
+        <v>0.2688</v>
       </c>
     </row>
     <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="13" t="inlineStr">
-        <is>
-          <t>1. AE-Specific Mode Imputation: Missing outc_cod values are filled with the most common outcome associated with that specific adverse event (pt_term) in the historical dataset (imputed 5,149 values in Obesity All, and 4,856 in Obesity Selected 4).</t>
-        </is>
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>Diabetes Selected 4 Drugs</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="n">
+        <v>342</v>
+      </c>
+      <c r="C13" s="8" t="n">
+        <v>116</v>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>33.92%</t>
+        </is>
+      </c>
+      <c r="E13" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="F13" s="7" t="inlineStr">
+        <is>
+          <t>Random Forest</t>
+        </is>
+      </c>
+      <c r="G13" s="10" t="n">
+        <v>0.9275</v>
+      </c>
+      <c r="H13" s="10" t="n">
+        <v>0.747</v>
       </c>
     </row>
     <row r="14" ht="18" customHeight="1">
-      <c r="A14" s="13" t="inlineStr">
-        <is>
-          <t>2. Clinical Indicator Fallback: Remaining missing values are imputed using fallback rules based on is_fatal (DE), severity_score &gt;= 4 (LT), severity_score &gt;= 3 (HO), is_serious (OT), or defaulting to OT.</t>
-        </is>
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Diabetes Selected 4 Drugs</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="n">
+        <v>342</v>
+      </c>
+      <c r="C14" s="4" t="n">
+        <v>116</v>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>33.92%</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="G14" s="6" t="n">
+        <v>0.9565</v>
+      </c>
+      <c r="H14" s="6" t="n">
+        <v>0.7454</v>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1">
-      <c r="A15" s="13" t="inlineStr">
-        <is>
-          <t>This resolved all missing entries to one of the 6 actual clinical outcomes: DE (Death), DS (Disability), HO (Hospitalization), LT (Life-Threatening), OT (Other Serious), and RI (Required Intervention).</t>
-        </is>
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>Diabetes Selected 4 Drugs</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="n">
+        <v>342</v>
+      </c>
+      <c r="C15" s="8" t="n">
+        <v>116</v>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>33.92%</t>
+        </is>
+      </c>
+      <c r="E15" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="F15" s="7" t="inlineStr">
+        <is>
+          <t>HANConv GNN</t>
+        </is>
+      </c>
+      <c r="G15" s="10" t="n">
+        <v>0.8406</v>
+      </c>
+      <c r="H15" s="10" t="n">
+        <v>0.5652</v>
       </c>
     </row>
     <row r="16"/>
     <row r="17" ht="22" customHeight="1">
       <c r="A17" s="11" t="inlineStr">
         <is>
+          <t>Imputation &amp; Preprocessing Methodology for outc_cod</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="12" t="inlineStr">
+        <is>
+          <t>The empty outcome values (5,933 in Obesity All, and 5,682 in Obesity Selected 4) were solved using a two-stage clinical imputation pipeline instead of simple deletion or filling with 'NS':</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="22" customHeight="1">
+      <c r="A19" s="13" t="inlineStr">
+        <is>
+          <t>1. AE-Specific Mode Imputation: Missing outc_cod values are filled with the most common outcome associated with that specific adverse event (pt_term) in the historical dataset (imputed 5,149 values in Obesity All, and 4,856 in Obesity Selected 4).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="13" t="inlineStr">
+        <is>
+          <t>2. Clinical Indicator Fallback: Remaining missing values are imputed using fallback rules based on is_fatal (DE), severity_score &gt;= 4 (LT), severity_score &gt;= 3 (HO), is_serious (OT), or defaulting to OT.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="13" t="inlineStr">
+        <is>
+          <t>This resolved all missing entries to one of the 6 actual clinical outcomes: DE (Death), DS (Disability), HO (Hospitalization), LT (Life-Threatening), OT (Other Serious), and RI (Required Intervention).</t>
+        </is>
+      </c>
+    </row>
+    <row r="22"/>
+    <row r="23">
+      <c r="A23" s="11" t="inlineStr">
+        <is>
           <t>FAERS Data Coverage: Year-Quarter Breakdown (fda_dt, 2021-2025)</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="14" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="14" t="inlineStr">
         <is>
           <t>Obesity All Drugs (14)</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="22" customHeight="1">
-      <c r="A19" s="15" t="inlineStr">
+    <row r="25" ht="20" customHeight="1">
+      <c r="A25" s="15" t="inlineStr">
         <is>
           <t>Year</t>
         </is>
       </c>
-      <c r="B19" s="15" t="inlineStr">
+      <c r="B25" s="15" t="inlineStr">
         <is>
           <t>Q1</t>
         </is>
       </c>
-      <c r="C19" s="15" t="inlineStr">
+      <c r="C25" s="15" t="inlineStr">
         <is>
           <t>Q2</t>
         </is>
       </c>
-      <c r="D19" s="15" t="inlineStr">
+      <c r="D25" s="15" t="inlineStr">
         <is>
           <t>Q3</t>
         </is>
       </c>
-      <c r="E19" s="15" t="inlineStr">
+      <c r="E25" s="15" t="inlineStr">
         <is>
           <t>Q4</t>
         </is>
       </c>
-      <c r="F19" s="15" t="inlineStr">
+      <c r="F25" s="15" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="16" t="n">
+    <row r="26">
+      <c r="A26" s="16" t="n">
         <v>2021</v>
       </c>
-      <c r="B20" s="16" t="n">
+      <c r="B26" s="16" t="n">
         <v>463</v>
       </c>
-      <c r="C20" s="16" t="n">
+      <c r="C26" s="16" t="n">
         <v>508</v>
       </c>
-      <c r="D20" s="16" t="n">
+      <c r="D26" s="16" t="n">
         <v>501</v>
       </c>
-      <c r="E20" s="16" t="n">
+      <c r="E26" s="16" t="n">
         <v>504</v>
       </c>
-      <c r="F20" s="16" t="n">
+      <c r="F26" s="16" t="n">
         <v>1976</v>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="9" t="n">
+    <row r="27" ht="20" customHeight="1">
+      <c r="A27" s="9" t="n">
         <v>2022</v>
       </c>
-      <c r="B21" s="9" t="n">
+      <c r="B27" s="9" t="n">
         <v>574</v>
       </c>
-      <c r="C21" s="9" t="n">
+      <c r="C27" s="9" t="n">
         <v>472</v>
       </c>
-      <c r="D21" s="9" t="n">
+      <c r="D27" s="9" t="n">
         <v>627</v>
       </c>
-      <c r="E21" s="9" t="n">
+      <c r="E27" s="9" t="n">
         <v>577</v>
       </c>
-      <c r="F21" s="9" t="n">
+      <c r="F27" s="9" t="n">
         <v>2250</v>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="16" t="n">
+    <row r="28" ht="22" customHeight="1">
+      <c r="A28" s="16" t="n">
         <v>2023</v>
       </c>
-      <c r="B22" s="16" t="n">
+      <c r="B28" s="16" t="n">
         <v>720</v>
       </c>
-      <c r="C22" s="16" t="n">
+      <c r="C28" s="16" t="n">
         <v>626</v>
       </c>
-      <c r="D22" s="16" t="n">
+      <c r="D28" s="16" t="n">
         <v>700</v>
       </c>
-      <c r="E22" s="16" t="n">
+      <c r="E28" s="16" t="n">
         <v>559</v>
       </c>
-      <c r="F22" s="16" t="n">
+      <c r="F28" s="16" t="n">
         <v>2605</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="9" t="n">
-        <v>2024</v>
-      </c>
-      <c r="B23" s="9" t="n">
-        <v>540</v>
-      </c>
-      <c r="C23" s="9" t="n">
-        <v>419</v>
-      </c>
-      <c r="D23" s="9" t="n">
-        <v>534</v>
-      </c>
-      <c r="E23" s="9" t="n">
-        <v>565</v>
-      </c>
-      <c r="F23" s="9" t="n">
-        <v>2058</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="16" t="n">
-        <v>2025</v>
-      </c>
-      <c r="B24" s="16" t="n">
-        <v>599</v>
-      </c>
-      <c r="C24" s="16" t="n">
-        <v>614</v>
-      </c>
-      <c r="D24" s="16" t="n">
-        <v>836</v>
-      </c>
-      <c r="E24" s="16" t="n">
-        <v>763</v>
-      </c>
-      <c r="F24" s="16" t="n">
-        <v>2812</v>
-      </c>
-    </row>
-    <row r="25" ht="20" customHeight="1">
-      <c r="A25" s="17" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="B25" s="18" t="n"/>
-      <c r="C25" s="18" t="n"/>
-      <c r="D25" s="18" t="n"/>
-      <c r="E25" s="18" t="n"/>
-      <c r="F25" s="17" t="n">
-        <v>11701</v>
-      </c>
-    </row>
-    <row r="26"/>
-    <row r="27" ht="20" customHeight="1">
-      <c r="A27" s="14" t="inlineStr">
-        <is>
-          <t>Obesity Selected 4 Drugs</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="22" customHeight="1">
-      <c r="A28" s="15" t="inlineStr">
-        <is>
-          <t>Year</t>
-        </is>
-      </c>
-      <c r="B28" s="15" t="inlineStr">
-        <is>
-          <t>Q1</t>
-        </is>
-      </c>
-      <c r="C28" s="15" t="inlineStr">
-        <is>
-          <t>Q2</t>
-        </is>
-      </c>
-      <c r="D28" s="15" t="inlineStr">
-        <is>
-          <t>Q3</t>
-        </is>
-      </c>
-      <c r="E28" s="15" t="inlineStr">
-        <is>
-          <t>Q4</t>
-        </is>
-      </c>
-      <c r="F28" s="15" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="9" t="n">
-        <v>2021</v>
+        <v>2024</v>
       </c>
       <c r="B29" s="9" t="n">
-        <v>431</v>
+        <v>540</v>
       </c>
       <c r="C29" s="9" t="n">
-        <v>469</v>
+        <v>419</v>
       </c>
       <c r="D29" s="9" t="n">
-        <v>472</v>
+        <v>534</v>
       </c>
       <c r="E29" s="9" t="n">
-        <v>463</v>
+        <v>565</v>
       </c>
       <c r="F29" s="9" t="n">
-        <v>1835</v>
+        <v>2058</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="16" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B30" s="16" t="n">
+        <v>599</v>
+      </c>
+      <c r="C30" s="16" t="n">
+        <v>614</v>
+      </c>
+      <c r="D30" s="16" t="n">
+        <v>836</v>
+      </c>
+      <c r="E30" s="16" t="n">
+        <v>763</v>
+      </c>
+      <c r="F30" s="16" t="n">
+        <v>2812</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="17" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B31" s="18" t="n"/>
+      <c r="C31" s="18" t="n"/>
+      <c r="D31" s="18" t="n"/>
+      <c r="E31" s="18" t="n"/>
+      <c r="F31" s="17" t="n">
+        <v>11701</v>
+      </c>
+    </row>
+    <row r="32"/>
+    <row r="33">
+      <c r="A33" s="14" t="inlineStr">
+        <is>
+          <t>Obesity Selected 4 Drugs</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="20" customHeight="1">
+      <c r="A34" s="15" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="B34" s="15" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="C34" s="15" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="D34" s="15" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="E34" s="15" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
+      <c r="F34" s="15" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="9" t="n">
+        <v>2021</v>
+      </c>
+      <c r="B35" s="9" t="n">
+        <v>431</v>
+      </c>
+      <c r="C35" s="9" t="n">
+        <v>469</v>
+      </c>
+      <c r="D35" s="9" t="n">
+        <v>472</v>
+      </c>
+      <c r="E35" s="9" t="n">
+        <v>463</v>
+      </c>
+      <c r="F35" s="9" t="n">
+        <v>1835</v>
+      </c>
+    </row>
+    <row r="36" ht="22" customHeight="1">
+      <c r="A36" s="16" t="n">
         <v>2022</v>
       </c>
-      <c r="B30" s="16" t="n">
+      <c r="B36" s="16" t="n">
         <v>544</v>
       </c>
-      <c r="C30" s="16" t="n">
+      <c r="C36" s="16" t="n">
         <v>447</v>
       </c>
-      <c r="D30" s="16" t="n">
+      <c r="D36" s="16" t="n">
         <v>585</v>
       </c>
-      <c r="E30" s="16" t="n">
+      <c r="E36" s="16" t="n">
         <v>529</v>
       </c>
-      <c r="F30" s="16" t="n">
+      <c r="F36" s="16" t="n">
         <v>2105</v>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="9" t="n">
+    <row r="37" ht="18" customHeight="1">
+      <c r="A37" s="9" t="n">
         <v>2023</v>
       </c>
-      <c r="B31" s="9" t="n">
+      <c r="B37" s="9" t="n">
         <v>676</v>
       </c>
-      <c r="C31" s="9" t="n">
+      <c r="C37" s="9" t="n">
         <v>572</v>
       </c>
-      <c r="D31" s="9" t="n">
+      <c r="D37" s="9" t="n">
         <v>631</v>
       </c>
-      <c r="E31" s="9" t="n">
+      <c r="E37" s="9" t="n">
         <v>520</v>
       </c>
-      <c r="F31" s="9" t="n">
+      <c r="F37" s="9" t="n">
         <v>2399</v>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="16" t="n">
+    <row r="38" ht="18" customHeight="1">
+      <c r="A38" s="16" t="n">
         <v>2024</v>
       </c>
-      <c r="B32" s="16" t="n">
+      <c r="B38" s="16" t="n">
         <v>491</v>
       </c>
-      <c r="C32" s="16" t="n">
+      <c r="C38" s="16" t="n">
         <v>385</v>
       </c>
-      <c r="D32" s="16" t="n">
+      <c r="D38" s="16" t="n">
         <v>482</v>
       </c>
-      <c r="E32" s="16" t="n">
+      <c r="E38" s="16" t="n">
         <v>518</v>
       </c>
-      <c r="F32" s="16" t="n">
+      <c r="F38" s="16" t="n">
         <v>1876</v>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="9" t="n">
+    <row r="39" ht="18" customHeight="1">
+      <c r="A39" s="9" t="n">
         <v>2025</v>
       </c>
-      <c r="B33" s="9" t="n">
+      <c r="B39" s="9" t="n">
         <v>542</v>
       </c>
-      <c r="C33" s="9" t="n">
+      <c r="C39" s="9" t="n">
         <v>550</v>
       </c>
-      <c r="D33" s="9" t="n">
+      <c r="D39" s="9" t="n">
         <v>727</v>
       </c>
-      <c r="E33" s="9" t="n">
+      <c r="E39" s="9" t="n">
         <v>667</v>
       </c>
-      <c r="F33" s="9" t="n">
+      <c r="F39" s="9" t="n">
         <v>2486</v>
       </c>
     </row>
-    <row r="34" ht="20" customHeight="1">
-      <c r="A34" s="17" t="inlineStr">
+    <row r="40" ht="18" customHeight="1">
+      <c r="A40" s="17" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B34" s="18" t="n"/>
-      <c r="C34" s="18" t="n"/>
-      <c r="D34" s="18" t="n"/>
-      <c r="E34" s="18" t="n"/>
-      <c r="F34" s="17" t="n">
+      <c r="B40" s="18" t="n"/>
+      <c r="C40" s="18" t="n"/>
+      <c r="D40" s="18" t="n"/>
+      <c r="E40" s="18" t="n"/>
+      <c r="F40" s="17" t="n">
         <v>10701</v>
       </c>
     </row>
-    <row r="35"/>
-    <row r="36" ht="22" customHeight="1">
-      <c r="A36" s="11" t="inlineStr">
+    <row r="41" ht="18" customHeight="1"/>
+    <row r="42">
+      <c r="A42" s="11" t="inlineStr">
         <is>
           <t>HANConv GNN Performance Analysis</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="18" customHeight="1">
-      <c r="A37" s="13" t="inlineStr">
+    <row r="43" ht="22" customHeight="1">
+      <c r="A43" s="13" t="inlineStr">
         <is>
           <t>The HANConv GNN achieves lower accuracy (~59-61%) and Macro-F1 (~12-13%) compared to XGBoost (94-95%). This is expected for the following reasons:</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="18" customHeight="1">
-      <c r="A38" s="13" t="inlineStr">
-        <is>
-          <t>1. Class Imbalance: OT (Other Serious) dominates ~60% of the data, while RI (Required Intervention) has only 3-5 samples. The GNN tends to predict the majority class.</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="18" customHeight="1">
-      <c r="A39" s="13" t="inlineStr">
-        <is>
-          <t>2. Graph Structure: With only 15-17 drug nodes and 1,600-1,726 ADR nodes, the heterogeneous graph is relatively sparse for HANConv to learn meaningful attention patterns.</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="18" customHeight="1">
-      <c r="A40" s="13" t="inlineStr">
-        <is>
-          <t>3. Tabular Data Strength: XGBoost and Random Forest excel on structured tabular features with categorical encoding, which is the natural format of FAERS pharmacovigilance data.</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="18" customHeight="1">
-      <c r="A41" s="13" t="inlineStr">
-        <is>
-          <t>4. Data is Complete: The low GNN performance is NOT a data issue. All 20 quarters (2021 Q1 through 2025 Q4) are fully represented in both datasets.</t>
-        </is>
-      </c>
-    </row>
-    <row r="42"/>
-    <row r="43" ht="22" customHeight="1">
-      <c r="A43" s="11" t="inlineStr">
-        <is>
-          <t>Strategies for Improving HANConv GNN Multiclass Performance</t>
         </is>
       </c>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="13" t="inlineStr">
         <is>
-          <t>To improve multiclass classification accuracy for graph neural networks in future work:</t>
+          <t>1. Class Imbalance: OT (Other Serious) dominates ~60% of the data, while RI (Required Intervention) has only 3-5 samples. The GNN tends to predict the majority class.</t>
         </is>
       </c>
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="13" t="inlineStr">
         <is>
-          <t>1. Introduce Semantic Node Features: Use pre-trained chemical fingerprint embeddings (e.g., PubChem fingerprints) for drug nodes and biomedical ontology embeddings (e.g., UMLS/MedDRA codes via BioBERT) for reaction (pt_term) nodes instead of degree-based initialization.</t>
+          <t>2. Graph Structure: With only 15-17 drug nodes and 1,600-1,726 ADR nodes, the heterogeneous graph is relatively sparse for HANConv to learn meaningful attention patterns.</t>
         </is>
       </c>
     </row>
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="13" t="inlineStr">
         <is>
-          <t>2. Class-Balanced Loss Functions: Deploy Class-Weighted Cross-Entropy or Focal Loss to heavily penalize errors on minority classes (e.g., RI, DS) and combat high class imbalance.</t>
+          <t>3. Tabular Data Strength: XGBoost and Random Forest excel on structured tabular features with categorical encoding, which is the natural format of FAERS pharmacovigilance data.</t>
         </is>
       </c>
     </row>
     <row r="47" ht="18" customHeight="1">
       <c r="A47" s="13" t="inlineStr">
         <is>
-          <t>3. Homogeneous Knowledge Bridges: Enrich graph topology by incorporating auxiliary homogeneous edges representing drug-drug chemical similarities and reaction-reaction clinical similarities.</t>
+          <t>4. Data is Complete: The low GNN performance is NOT a data issue. All 20 quarters (2021 Q1 through 2025 Q4) are fully represented in both datasets.</t>
         </is>
       </c>
     </row>
@@ -1255,116 +1411,151 @@
     <row r="49" ht="22" customHeight="1">
       <c r="A49" s="11" t="inlineStr">
         <is>
-          <t>Scientific Paper Framing (Recommended LaTeX Paragraph)</t>
+          <t>Strategies for Improving HANConv GNN Multiclass Performance</t>
         </is>
       </c>
     </row>
     <row r="50" ht="16" customHeight="1">
       <c r="A50" s="13" t="inlineStr">
         <is>
-          <t>To justify the model choice in your journal manuscript, copy and insert the following paragraph:</t>
+          <t>To improve multiclass classification accuracy for graph neural networks in future work:</t>
         </is>
       </c>
     </row>
     <row r="51" ht="16" customHeight="1">
-      <c r="A51" s="19" t="inlineStr">
-        <is>
-          <t>--------------------------------------------------------------------------------------------------------------------------------------------------------</t>
+      <c r="A51" s="13" t="inlineStr">
+        <is>
+          <t>1. Introduce Semantic Node Features: Use pre-trained chemical fingerprint embeddings (e.g., PubChem fingerprints) for drug nodes and biomedical ontology embeddings (e.g., UMLS/MedDRA codes via BioBERT) for reaction (pt_term) nodes instead of degree-based initialization.</t>
         </is>
       </c>
     </row>
     <row r="52" ht="16" customHeight="1">
-      <c r="A52" s="20" t="inlineStr">
-        <is>
-          <t>\subsection{Sub-Cohort Analysis and Tabular Model Justification}</t>
+      <c r="A52" s="13" t="inlineStr">
+        <is>
+          <t>2. Class-Balanced Loss Functions: Deploy Class-Weighted Cross-Entropy or Focal Loss to heavily penalize errors on minority classes (e.g., RI, DS) and combat high class imbalance.</t>
         </is>
       </c>
     </row>
     <row r="53" ht="16" customHeight="1">
       <c r="A53" s="13" t="inlineStr">
         <is>
-          <t>While the global signal detection pipeline relies on the scale and structural learning capabilities of the heterogeneous</t>
-        </is>
-      </c>
-    </row>
-    <row r="54" ht="16" customHeight="1">
-      <c r="A54" s="19" t="inlineStr">
-        <is>
-          <t>HANConv Graph Neural Network (GNN), local sub-cohort analyses---specifically anti-obesity and anti-diabetic cohorts---</t>
-        </is>
-      </c>
-    </row>
+          <t>3. Homogeneous Knowledge Bridges: Enrich graph topology by incorporating auxiliary homogeneous edges representing drug-drug chemical similarities and reaction-reaction clinical similarities.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="16" customHeight="1"/>
     <row r="55" ht="16" customHeight="1">
-      <c r="A55" s="13" t="inlineStr">
-        <is>
-          <t>present distinct structural characteristics. When restricting the reporting network to a narrow subset of anti-obesity agents</t>
+      <c r="A55" s="11" t="inlineStr">
+        <is>
+          <t>Scientific Paper Framing (Recommended LaTeX Paragraph)</t>
         </is>
       </c>
     </row>
     <row r="56" ht="16" customHeight="1">
       <c r="A56" s="13" t="inlineStr">
         <is>
-          <t>(e.g., Semaglutide, Liraglutide, Tirzepatide), the resulting subgraph becomes highly sparse, with a restricted neighborhood</t>
+          <t>To justify the model choice in your journal manuscript, copy and insert the following paragraph:</t>
         </is>
       </c>
     </row>
     <row r="57" ht="16" customHeight="1">
-      <c r="A57" s="13" t="inlineStr">
-        <is>
-          <t>size that limits the message-passing efficiency of graph attention mechanisms. To overcome this localized sparsity, we deployed</t>
+      <c r="A57" s="19" t="inlineStr">
+        <is>
+          <t>--------------------------------------------------------------------------------------------------------------------------------------------------------</t>
         </is>
       </c>
     </row>
     <row r="58" ht="16" customHeight="1">
-      <c r="A58" s="13" t="inlineStr">
-        <is>
-          <t>tabular gradient-boosted decision trees (XGBoost) alongside the GNN. Empirically, XGBoost demonstrated superior multiclass</t>
+      <c r="A58" s="20" t="inlineStr">
+        <is>
+          <t>\subsection{Sub-Cohort Analysis and Tabular Model Justification}</t>
         </is>
       </c>
     </row>
     <row r="59" ht="16" customHeight="1">
       <c r="A59" s="13" t="inlineStr">
         <is>
-          <t>outcome prediction accuracy (94.2% to 94.7%) compared to the HANConv GNN (59.6% to 61.2%). Tabular classifiers excel in this</t>
+          <t>While the global signal detection pipeline relies on the scale and structural learning capabilities of the heterogeneous</t>
         </is>
       </c>
     </row>
     <row r="60" ht="16" customHeight="1">
-      <c r="A60" s="13" t="inlineStr">
-        <is>
-          <t>sub-cohort because the prediction task depends heavily on dense, report-level features (e.g., patient age, weight, administered</t>
+      <c r="A60" s="19" t="inlineStr">
+        <is>
+          <t>HANConv Graph Neural Network (GNN), local sub-cohort analyses---specifically anti-obesity and anti-diabetic cohorts---</t>
         </is>
       </c>
     </row>
     <row r="61" ht="16" customHeight="1">
       <c r="A61" s="13" t="inlineStr">
         <is>
-          <t>dose, and normalized drug sequence roles) rather than wider topological reporting networks. Consequently, we present XGBoost</t>
+          <t>present distinct structural characteristics. When restricting the reporting network to a narrow subset of anti-obesity agents</t>
         </is>
       </c>
     </row>
     <row r="62" ht="16" customHeight="1">
       <c r="A62" s="13" t="inlineStr">
         <is>
-          <t>as the primary predictive engine for the anti-obesity cohort, while maintaining the HANConv GNN architecture for global,</t>
+          <t>(e.g., Semaglutide, Liraglutide, Tirzepatide), the resulting subgraph becomes highly sparse, with a restricted neighborhood</t>
         </is>
       </c>
     </row>
     <row r="63" ht="16" customHeight="1">
       <c r="A63" s="13" t="inlineStr">
         <is>
+          <t>size that limits the message-passing efficiency of graph attention mechanisms. To overcome this localized sparsity, we deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="16" customHeight="1">
+      <c r="A64" s="13" t="inlineStr">
+        <is>
+          <t>tabular gradient-boosted decision trees (XGBoost) alongside the GNN. Empirically, XGBoost demonstrated superior multiclass</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="13" t="inlineStr">
+        <is>
+          <t>outcome prediction accuracy (94.2% to 94.7%) compared to the HANConv GNN (59.6% to 61.2%). Tabular classifiers excel in this</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="13" t="inlineStr">
+        <is>
+          <t>sub-cohort because the prediction task depends heavily on dense, report-level features (e.g., patient age, weight, administered</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="13" t="inlineStr">
+        <is>
+          <t>dose, and normalized drug sequence roles) rather than wider topological reporting networks. Consequently, we present XGBoost</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="13" t="inlineStr">
+        <is>
+          <t>as the primary predictive engine for the anti-obesity cohort, while maintaining the HANConv GNN architecture for global,</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="13" t="inlineStr">
+        <is>
           <t>multi-drug signal detection where network topology is the dominant feature.</t>
         </is>
       </c>
     </row>
-    <row r="64" ht="16" customHeight="1">
-      <c r="A64" s="19" t="inlineStr">
+    <row r="70">
+      <c r="A70" s="19" t="inlineStr">
         <is>
           <t>--------------------------------------------------------------------------------------------------------------------------------------------------------</t>
         </is>
       </c>
     </row>
-    <row r="65"/>
   </sheetData>
   <mergeCells count="36">
     <mergeCell ref="A39:H39"/>

</xml_diff>

<commit_message>
Populate all missing Year-Quarter breakdown tables and metrics in comparison sheet
</commit_message>
<xml_diff>
--- a/dataset/15 Columns Leakage/ML_Multiclass_Model_Comparison_Results.xlsx
+++ b/dataset/15 Columns Leakage/ML_Multiclass_Model_Comparison_Results.xlsx
@@ -117,7 +117,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -138,6 +138,50 @@
       <bottom style="thin">
         <color rgb="00D3D3D3"/>
       </bottom>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D3D3D3"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D3D3D3"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D3D3D3"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D3D3D3"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D3D3D3"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D3D3D3"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D3D3D3"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D3D3D3"/>
+      </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
@@ -566,7 +610,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H70"/>
+  <dimension ref="A1:H88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -1013,7 +1057,6 @@
         <v>0.5652</v>
       </c>
     </row>
-    <row r="16"/>
     <row r="17" ht="22" customHeight="1">
       <c r="A17" s="11" t="inlineStr">
         <is>
@@ -1049,7 +1092,6 @@
         </is>
       </c>
     </row>
-    <row r="22"/>
     <row r="23">
       <c r="A23" s="11" t="inlineStr">
         <is>
@@ -1120,19 +1162,19 @@
       <c r="A27" s="9" t="n">
         <v>2022</v>
       </c>
-      <c r="B27" s="9" t="n">
+      <c r="B27" t="n">
         <v>574</v>
       </c>
-      <c r="C27" s="9" t="n">
+      <c r="C27" t="n">
         <v>472</v>
       </c>
-      <c r="D27" s="9" t="n">
+      <c r="D27" t="n">
         <v>627</v>
       </c>
-      <c r="E27" s="9" t="n">
+      <c r="E27" t="n">
         <v>577</v>
       </c>
-      <c r="F27" s="9" t="n">
+      <c r="F27" t="n">
         <v>2250</v>
       </c>
     </row>
@@ -1202,15 +1244,22 @@
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B31" s="18" t="n"/>
-      <c r="C31" s="18" t="n"/>
-      <c r="D31" s="18" t="n"/>
-      <c r="E31" s="18" t="n"/>
+      <c r="B31" s="18" t="n">
+        <v>2896</v>
+      </c>
+      <c r="C31" s="18" t="n">
+        <v>2639</v>
+      </c>
+      <c r="D31" s="18" t="n">
+        <v>3198</v>
+      </c>
+      <c r="E31" s="18" t="n">
+        <v>2968</v>
+      </c>
       <c r="F31" s="17" t="n">
         <v>11701</v>
       </c>
     </row>
-    <row r="32"/>
     <row r="33">
       <c r="A33" s="14" t="inlineStr">
         <is>
@@ -1274,19 +1323,19 @@
       <c r="A36" s="16" t="n">
         <v>2022</v>
       </c>
-      <c r="B36" s="16" t="n">
+      <c r="B36" t="n">
         <v>544</v>
       </c>
-      <c r="C36" s="16" t="n">
+      <c r="C36" t="n">
         <v>447</v>
       </c>
-      <c r="D36" s="16" t="n">
+      <c r="D36" t="n">
         <v>585</v>
       </c>
-      <c r="E36" s="16" t="n">
+      <c r="E36" t="n">
         <v>529</v>
       </c>
-      <c r="F36" s="16" t="n">
+      <c r="F36" t="n">
         <v>2105</v>
       </c>
     </row>
@@ -1294,19 +1343,19 @@
       <c r="A37" s="9" t="n">
         <v>2023</v>
       </c>
-      <c r="B37" s="9" t="n">
+      <c r="B37" t="n">
         <v>676</v>
       </c>
-      <c r="C37" s="9" t="n">
+      <c r="C37" t="n">
         <v>572</v>
       </c>
-      <c r="D37" s="9" t="n">
+      <c r="D37" t="n">
         <v>631</v>
       </c>
-      <c r="E37" s="9" t="n">
+      <c r="E37" t="n">
         <v>520</v>
       </c>
-      <c r="F37" s="9" t="n">
+      <c r="F37" t="n">
         <v>2399</v>
       </c>
     </row>
@@ -1314,19 +1363,19 @@
       <c r="A38" s="16" t="n">
         <v>2024</v>
       </c>
-      <c r="B38" s="16" t="n">
+      <c r="B38" t="n">
         <v>491</v>
       </c>
-      <c r="C38" s="16" t="n">
+      <c r="C38" t="n">
         <v>385</v>
       </c>
-      <c r="D38" s="16" t="n">
+      <c r="D38" t="n">
         <v>482</v>
       </c>
-      <c r="E38" s="16" t="n">
+      <c r="E38" t="n">
         <v>518</v>
       </c>
-      <c r="F38" s="16" t="n">
+      <c r="F38" t="n">
         <v>1876</v>
       </c>
     </row>
@@ -1334,19 +1383,19 @@
       <c r="A39" s="9" t="n">
         <v>2025</v>
       </c>
-      <c r="B39" s="9" t="n">
+      <c r="B39" t="n">
         <v>542</v>
       </c>
-      <c r="C39" s="9" t="n">
+      <c r="C39" t="n">
         <v>550</v>
       </c>
-      <c r="D39" s="9" t="n">
+      <c r="D39" t="n">
         <v>727</v>
       </c>
-      <c r="E39" s="9" t="n">
+      <c r="E39" t="n">
         <v>667</v>
       </c>
-      <c r="F39" s="9" t="n">
+      <c r="F39" t="n">
         <v>2486</v>
       </c>
     </row>
@@ -1356,244 +1405,571 @@
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B40" s="18" t="n"/>
-      <c r="C40" s="18" t="n"/>
-      <c r="D40" s="18" t="n"/>
-      <c r="E40" s="18" t="n"/>
-      <c r="F40" s="17" t="n">
+      <c r="B40" t="n">
+        <v>2685</v>
+      </c>
+      <c r="C40" t="n">
+        <v>2423</v>
+      </c>
+      <c r="D40" t="n">
+        <v>2897</v>
+      </c>
+      <c r="E40" t="n">
+        <v>2696</v>
+      </c>
+      <c r="F40" t="n">
         <v>10701</v>
       </c>
     </row>
     <row r="41" ht="18" customHeight="1"/>
     <row r="42">
-      <c r="A42" s="11" t="inlineStr">
+      <c r="A42" s="14" t="inlineStr">
+        <is>
+          <t>Diabetes All Drugs (10)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="22" customHeight="1">
+      <c r="A43" s="15" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="B43" s="15" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="C43" s="15" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="D43" s="15" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="E43" s="15" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
+      <c r="F43" s="15" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="18" customHeight="1">
+      <c r="A44" s="9" t="n">
+        <v>2021</v>
+      </c>
+      <c r="B44" s="9" t="n">
+        <v>235</v>
+      </c>
+      <c r="C44" s="9" t="n">
+        <v>240</v>
+      </c>
+      <c r="D44" s="9" t="n">
+        <v>202</v>
+      </c>
+      <c r="E44" s="9" t="n">
+        <v>263</v>
+      </c>
+      <c r="F44" s="9" t="n">
+        <v>940</v>
+      </c>
+    </row>
+    <row r="45" ht="18" customHeight="1">
+      <c r="A45" s="16" t="n">
+        <v>2022</v>
+      </c>
+      <c r="B45" t="n">
+        <v>262</v>
+      </c>
+      <c r="C45" t="n">
+        <v>210</v>
+      </c>
+      <c r="D45" t="n">
+        <v>255</v>
+      </c>
+      <c r="E45" t="n">
+        <v>256</v>
+      </c>
+      <c r="F45" t="n">
+        <v>983</v>
+      </c>
+    </row>
+    <row r="46" ht="18" customHeight="1">
+      <c r="A46" s="9" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B46" t="n">
+        <v>275</v>
+      </c>
+      <c r="C46" t="n">
+        <v>263</v>
+      </c>
+      <c r="D46" t="n">
+        <v>302</v>
+      </c>
+      <c r="E46" t="n">
+        <v>287</v>
+      </c>
+      <c r="F46" t="n">
+        <v>1127</v>
+      </c>
+    </row>
+    <row r="47" ht="18" customHeight="1">
+      <c r="A47" s="16" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B47" t="n">
+        <v>254</v>
+      </c>
+      <c r="C47" t="n">
+        <v>186</v>
+      </c>
+      <c r="D47" t="n">
+        <v>242</v>
+      </c>
+      <c r="E47" t="n">
+        <v>241</v>
+      </c>
+      <c r="F47" t="n">
+        <v>923</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="9" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B48" t="n">
+        <v>240</v>
+      </c>
+      <c r="C48" t="n">
+        <v>279</v>
+      </c>
+      <c r="D48" t="n">
+        <v>362</v>
+      </c>
+      <c r="E48" t="n">
+        <v>354</v>
+      </c>
+      <c r="F48" t="n">
+        <v>1235</v>
+      </c>
+    </row>
+    <row r="49" ht="22" customHeight="1">
+      <c r="A49" s="17" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>1266</v>
+      </c>
+      <c r="C49" t="n">
+        <v>1178</v>
+      </c>
+      <c r="D49" t="n">
+        <v>1363</v>
+      </c>
+      <c r="E49" t="n">
+        <v>1401</v>
+      </c>
+      <c r="F49" t="n">
+        <v>5208</v>
+      </c>
+    </row>
+    <row r="50" ht="16" customHeight="1"/>
+    <row r="51" ht="16" customHeight="1">
+      <c r="A51" s="14" t="inlineStr">
+        <is>
+          <t>Diabetes Selected 4 Drugs</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="16" customHeight="1">
+      <c r="A52" s="15" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="B52" s="15" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="C52" s="15" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="D52" s="15" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="E52" s="15" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
+      <c r="F52" s="15" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="16" customHeight="1">
+      <c r="A53" s="9" t="n">
+        <v>2021</v>
+      </c>
+      <c r="B53" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="C53" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D53" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E53" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F53" s="9" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="54" ht="16" customHeight="1">
+      <c r="A54" s="16" t="n">
+        <v>2022</v>
+      </c>
+      <c r="B54" t="n">
+        <v>3</v>
+      </c>
+      <c r="C54" t="n">
+        <v>10</v>
+      </c>
+      <c r="D54" t="n">
+        <v>4</v>
+      </c>
+      <c r="E54" t="n">
+        <v>4</v>
+      </c>
+      <c r="F54" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="55" ht="16" customHeight="1">
+      <c r="A55" s="9" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B55" t="n">
+        <v>14</v>
+      </c>
+      <c r="C55" t="n">
+        <v>21</v>
+      </c>
+      <c r="D55" t="n">
+        <v>33</v>
+      </c>
+      <c r="E55" t="n">
+        <v>8</v>
+      </c>
+      <c r="F55" t="n">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="56" ht="16" customHeight="1">
+      <c r="A56" s="16" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B56" t="n">
+        <v>22</v>
+      </c>
+      <c r="C56" t="n">
+        <v>24</v>
+      </c>
+      <c r="D56" t="n">
+        <v>18</v>
+      </c>
+      <c r="E56" t="n">
+        <v>19</v>
+      </c>
+      <c r="F56" t="n">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="57" ht="16" customHeight="1">
+      <c r="A57" s="9" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B57" t="n">
+        <v>30</v>
+      </c>
+      <c r="C57" t="n">
+        <v>18</v>
+      </c>
+      <c r="D57" t="n">
+        <v>62</v>
+      </c>
+      <c r="E57" t="n">
+        <v>46</v>
+      </c>
+      <c r="F57" t="n">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="58" ht="16" customHeight="1">
+      <c r="A58" s="17" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>73</v>
+      </c>
+      <c r="C58" t="n">
+        <v>72</v>
+      </c>
+      <c r="D58" t="n">
+        <v>117</v>
+      </c>
+      <c r="E58" t="n">
+        <v>80</v>
+      </c>
+      <c r="F58" t="n">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="59" ht="16" customHeight="1"/>
+    <row r="60" ht="16" customHeight="1">
+      <c r="A60" s="11" t="inlineStr">
         <is>
           <t>HANConv GNN Performance Analysis</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="22" customHeight="1">
-      <c r="A43" s="13" t="inlineStr">
-        <is>
-          <t>The HANConv GNN achieves lower accuracy (~59-61%) and Macro-F1 (~12-13%) compared to XGBoost (94-95%). This is expected for the following reasons:</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="18" customHeight="1">
-      <c r="A44" s="13" t="inlineStr">
-        <is>
-          <t>1. Class Imbalance: OT (Other Serious) dominates ~60% of the data, while RI (Required Intervention) has only 3-5 samples. The GNN tends to predict the majority class.</t>
-        </is>
-      </c>
-    </row>
-    <row r="45" ht="18" customHeight="1">
-      <c r="A45" s="13" t="inlineStr">
-        <is>
-          <t>2. Graph Structure: With only 15-17 drug nodes and 1,600-1,726 ADR nodes, the heterogeneous graph is relatively sparse for HANConv to learn meaningful attention patterns.</t>
-        </is>
-      </c>
-    </row>
-    <row r="46" ht="18" customHeight="1">
-      <c r="A46" s="13" t="inlineStr">
-        <is>
-          <t>3. Tabular Data Strength: XGBoost and Random Forest excel on structured tabular features with categorical encoding, which is the natural format of FAERS pharmacovigilance data.</t>
-        </is>
-      </c>
-    </row>
-    <row r="47" ht="18" customHeight="1">
-      <c r="A47" s="13" t="inlineStr">
-        <is>
-          <t>4. Data is Complete: The low GNN performance is NOT a data issue. All 20 quarters (2021 Q1 through 2025 Q4) are fully represented in both datasets.</t>
-        </is>
-      </c>
-    </row>
-    <row r="48"/>
-    <row r="49" ht="22" customHeight="1">
-      <c r="A49" s="11" t="inlineStr">
-        <is>
-          <t>Strategies for Improving HANConv GNN Multiclass Performance</t>
-        </is>
-      </c>
-    </row>
-    <row r="50" ht="16" customHeight="1">
-      <c r="A50" s="13" t="inlineStr">
-        <is>
-          <t>To improve multiclass classification accuracy for graph neural networks in future work:</t>
-        </is>
-      </c>
-    </row>
-    <row r="51" ht="16" customHeight="1">
-      <c r="A51" s="13" t="inlineStr">
-        <is>
-          <t>1. Introduce Semantic Node Features: Use pre-trained chemical fingerprint embeddings (e.g., PubChem fingerprints) for drug nodes and biomedical ontology embeddings (e.g., UMLS/MedDRA codes via BioBERT) for reaction (pt_term) nodes instead of degree-based initialization.</t>
-        </is>
-      </c>
-    </row>
-    <row r="52" ht="16" customHeight="1">
-      <c r="A52" s="13" t="inlineStr">
-        <is>
-          <t>2. Class-Balanced Loss Functions: Deploy Class-Weighted Cross-Entropy or Focal Loss to heavily penalize errors on minority classes (e.g., RI, DS) and combat high class imbalance.</t>
-        </is>
-      </c>
-    </row>
-    <row r="53" ht="16" customHeight="1">
-      <c r="A53" s="13" t="inlineStr">
-        <is>
-          <t>3. Homogeneous Knowledge Bridges: Enrich graph topology by incorporating auxiliary homogeneous edges representing drug-drug chemical similarities and reaction-reaction clinical similarities.</t>
-        </is>
-      </c>
-    </row>
-    <row r="54" ht="16" customHeight="1"/>
-    <row r="55" ht="16" customHeight="1">
-      <c r="A55" s="11" t="inlineStr">
-        <is>
-          <t>Scientific Paper Framing (Recommended LaTeX Paragraph)</t>
-        </is>
-      </c>
-    </row>
-    <row r="56" ht="16" customHeight="1">
-      <c r="A56" s="13" t="inlineStr">
-        <is>
-          <t>To justify the model choice in your journal manuscript, copy and insert the following paragraph:</t>
-        </is>
-      </c>
-    </row>
-    <row r="57" ht="16" customHeight="1">
-      <c r="A57" s="19" t="inlineStr">
-        <is>
-          <t>--------------------------------------------------------------------------------------------------------------------------------------------------------</t>
-        </is>
-      </c>
-    </row>
-    <row r="58" ht="16" customHeight="1">
-      <c r="A58" s="20" t="inlineStr">
-        <is>
-          <t>\subsection{Sub-Cohort Analysis and Tabular Model Justification}</t>
-        </is>
-      </c>
-    </row>
-    <row r="59" ht="16" customHeight="1">
-      <c r="A59" s="13" t="inlineStr">
-        <is>
-          <t>While the global signal detection pipeline relies on the scale and structural learning capabilities of the heterogeneous</t>
-        </is>
-      </c>
-    </row>
-    <row r="60" ht="16" customHeight="1">
-      <c r="A60" s="19" t="inlineStr">
-        <is>
-          <t>HANConv Graph Neural Network (GNN), local sub-cohort analyses---specifically anti-obesity and anti-diabetic cohorts---</t>
         </is>
       </c>
     </row>
     <row r="61" ht="16" customHeight="1">
       <c r="A61" s="13" t="inlineStr">
         <is>
-          <t>present distinct structural characteristics. When restricting the reporting network to a narrow subset of anti-obesity agents</t>
+          <t>The HANConv GNN achieves lower accuracy (~59-61%) and Macro-F1 (~12-13%) compared to XGBoost (94-95%). This is expected for the following reasons:</t>
         </is>
       </c>
     </row>
     <row r="62" ht="16" customHeight="1">
       <c r="A62" s="13" t="inlineStr">
         <is>
-          <t>(e.g., Semaglutide, Liraglutide, Tirzepatide), the resulting subgraph becomes highly sparse, with a restricted neighborhood</t>
+          <t>1. Class Imbalance: OT (Other Serious) dominates ~60% of the data, while RI (Required Intervention) has only 3-5 samples. The GNN tends to predict the majority class.</t>
         </is>
       </c>
     </row>
     <row r="63" ht="16" customHeight="1">
       <c r="A63" s="13" t="inlineStr">
         <is>
-          <t>size that limits the message-passing efficiency of graph attention mechanisms. To overcome this localized sparsity, we deployed</t>
+          <t>2. Graph Structure: With only 15-17 drug nodes and 1,600-1,726 ADR nodes, the heterogeneous graph is relatively sparse for HANConv to learn meaningful attention patterns.</t>
         </is>
       </c>
     </row>
     <row r="64" ht="16" customHeight="1">
       <c r="A64" s="13" t="inlineStr">
         <is>
-          <t>tabular gradient-boosted decision trees (XGBoost) alongside the GNN. Empirically, XGBoost demonstrated superior multiclass</t>
+          <t>3. Tabular Data Strength: XGBoost and Random Forest excel on structured tabular features with categorical encoding, which is the natural format of FAERS pharmacovigilance data.</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="13" t="inlineStr">
         <is>
-          <t>outcome prediction accuracy (94.2% to 94.7%) compared to the HANConv GNN (59.6% to 61.2%). Tabular classifiers excel in this</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="13" t="inlineStr">
-        <is>
-          <t>sub-cohort because the prediction task depends heavily on dense, report-level features (e.g., patient age, weight, administered</t>
-        </is>
-      </c>
-    </row>
+          <t>4. Data is Complete: The low GNN performance is NOT a data issue. All 20 quarters (2021 Q1 through 2025 Q4) are fully represented in both datasets.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66"/>
     <row r="67">
-      <c r="A67" s="13" t="inlineStr">
-        <is>
-          <t>dose, and normalized drug sequence roles) rather than wider topological reporting networks. Consequently, we present XGBoost</t>
+      <c r="A67" s="11" t="inlineStr">
+        <is>
+          <t>Strategies for Improving HANConv GNN Multiclass Performance</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="13" t="inlineStr">
         <is>
-          <t>as the primary predictive engine for the anti-obesity cohort, while maintaining the HANConv GNN architecture for global,</t>
+          <t>To improve multiclass classification accuracy for graph neural networks in future work:</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="13" t="inlineStr">
         <is>
+          <t>1. Introduce Semantic Node Features: Use pre-trained chemical fingerprint embeddings (e.g., PubChem fingerprints) for drug nodes and biomedical ontology embeddings (e.g., UMLS/MedDRA codes via BioBERT) for reaction (pt_term) nodes instead of degree-based initialization.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="13" t="inlineStr">
+        <is>
+          <t>2. Class-Balanced Loss Functions: Deploy Class-Weighted Cross-Entropy or Focal Loss to heavily penalize errors on minority classes (e.g., RI, DS) and combat high class imbalance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="13" t="inlineStr">
+        <is>
+          <t>3. Homogeneous Knowledge Bridges: Enrich graph topology by incorporating auxiliary homogeneous edges representing drug-drug chemical similarities and reaction-reaction clinical similarities.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72"/>
+    <row r="73">
+      <c r="A73" s="11" t="inlineStr">
+        <is>
+          <t>Scientific Paper Framing (Recommended LaTeX Paragraph)</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="13" t="inlineStr">
+        <is>
+          <t>To justify the model choice in your journal manuscript, copy and insert the following paragraph:</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="19" t="inlineStr">
+        <is>
+          <t>--------------------------------------------------------------------------------------------------------------------------------------------------------</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="20" t="inlineStr">
+        <is>
+          <t>\subsection{Sub-Cohort Analysis and Tabular Model Justification}</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="13" t="inlineStr">
+        <is>
+          <t>While the global signal detection pipeline relies on the scale and structural learning capabilities of the heterogeneous</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="19" t="inlineStr">
+        <is>
+          <t>HANConv Graph Neural Network (GNN), local sub-cohort analyses---specifically anti-obesity and anti-diabetic cohorts---</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="13" t="inlineStr">
+        <is>
+          <t>present distinct structural characteristics. When restricting the reporting network to a narrow subset of anti-obesity agents</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="13" t="inlineStr">
+        <is>
+          <t>(e.g., Semaglutide, Liraglutide, Tirzepatide), the resulting subgraph becomes highly sparse, with a restricted neighborhood</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="13" t="inlineStr">
+        <is>
+          <t>size that limits the message-passing efficiency of graph attention mechanisms. To overcome this localized sparsity, we deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="13" t="inlineStr">
+        <is>
+          <t>tabular gradient-boosted decision trees (XGBoost) alongside the GNN. Empirically, XGBoost demonstrated superior multiclass</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="13" t="inlineStr">
+        <is>
+          <t>outcome prediction accuracy (94.2% to 94.7%) compared to the HANConv GNN (59.6% to 61.2%). Tabular classifiers excel in this</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="13" t="inlineStr">
+        <is>
+          <t>sub-cohort because the prediction task depends heavily on dense, report-level features (e.g., patient age, weight, administered</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="13" t="inlineStr">
+        <is>
+          <t>dose, and normalized drug sequence roles) rather than wider topological reporting networks. Consequently, we present XGBoost</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="13" t="inlineStr">
+        <is>
+          <t>as the primary predictive engine for the anti-obesity cohort, while maintaining the HANConv GNN architecture for global,</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="13" t="inlineStr">
+        <is>
           <t>multi-drug signal detection where network topology is the dominant feature.</t>
         </is>
       </c>
     </row>
-    <row r="70">
-      <c r="A70" s="19" t="inlineStr">
+    <row r="88">
+      <c r="A88" s="19" t="inlineStr">
         <is>
           <t>--------------------------------------------------------------------------------------------------------------------------------------------------------</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="36">
-    <mergeCell ref="A39:H39"/>
-    <mergeCell ref="A15:H15"/>
-    <mergeCell ref="A59:H59"/>
+  <mergeCells count="31">
+    <mergeCell ref="A67:H67"/>
+    <mergeCell ref="A77:H77"/>
+    <mergeCell ref="A24:H24"/>
+    <mergeCell ref="A73:H73"/>
     <mergeCell ref="A51:H51"/>
     <mergeCell ref="A64:H64"/>
-    <mergeCell ref="A60:H60"/>
-    <mergeCell ref="A36:H36"/>
-    <mergeCell ref="A11:H11"/>
-    <mergeCell ref="A49:H49"/>
-    <mergeCell ref="A45:H45"/>
+    <mergeCell ref="A82:H82"/>
     <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A79:H79"/>
     <mergeCell ref="A61:H61"/>
-    <mergeCell ref="A54:H54"/>
-    <mergeCell ref="A41:H41"/>
-    <mergeCell ref="A46:H46"/>
-    <mergeCell ref="A37:H37"/>
-    <mergeCell ref="A27:H27"/>
-    <mergeCell ref="A12:H12"/>
+    <mergeCell ref="A70:H70"/>
+    <mergeCell ref="A78:H78"/>
+    <mergeCell ref="A69:H69"/>
+    <mergeCell ref="A65:H65"/>
+    <mergeCell ref="A80:H80"/>
+    <mergeCell ref="A75:H75"/>
+    <mergeCell ref="A74:H74"/>
     <mergeCell ref="A18:H18"/>
-    <mergeCell ref="A50:H50"/>
-    <mergeCell ref="A56:H56"/>
-    <mergeCell ref="A55:H55"/>
-    <mergeCell ref="A57:H57"/>
-    <mergeCell ref="A14:H14"/>
-    <mergeCell ref="A47:H47"/>
+    <mergeCell ref="A21:H21"/>
+    <mergeCell ref="A71:H71"/>
+    <mergeCell ref="A42:H42"/>
+    <mergeCell ref="A76:H76"/>
+    <mergeCell ref="A23:H23"/>
     <mergeCell ref="A17:H17"/>
     <mergeCell ref="A62:H62"/>
-    <mergeCell ref="A53:H53"/>
-    <mergeCell ref="A43:H43"/>
-    <mergeCell ref="A38:H38"/>
+    <mergeCell ref="A20:H20"/>
+    <mergeCell ref="A81:H81"/>
     <mergeCell ref="A63:H63"/>
-    <mergeCell ref="A52:H52"/>
-    <mergeCell ref="A13:H13"/>
-    <mergeCell ref="A44:H44"/>
-    <mergeCell ref="A58:H58"/>
-    <mergeCell ref="A40:H40"/>
+    <mergeCell ref="A72:H72"/>
+    <mergeCell ref="A68:H68"/>
+    <mergeCell ref="A19:H19"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix year-quarter breakdown table column misalignment by recreating merged cell ranges from scratch
</commit_message>
<xml_diff>
--- a/dataset/15 Columns Leakage/ML_Multiclass_Model_Comparison_Results.xlsx
+++ b/dataset/15 Columns Leakage/ML_Multiclass_Model_Comparison_Results.xlsx
@@ -187,7 +187,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -245,6 +245,8 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -610,7 +612,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H88"/>
+  <dimension ref="A1:H106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -1747,198 +1749,390 @@
     </row>
     <row r="59" ht="16" customHeight="1"/>
     <row r="60" ht="16" customHeight="1">
-      <c r="A60" s="11" t="inlineStr">
+      <c r="A60" s="14" t="inlineStr">
+        <is>
+          <t>Diabetes All Drugs (10)</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="16" customHeight="1">
+      <c r="A61" s="15" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="B61" s="21" t="n"/>
+      <c r="C61" s="21" t="n"/>
+      <c r="D61" s="21" t="n"/>
+      <c r="E61" s="21" t="n"/>
+      <c r="F61" s="21" t="n"/>
+      <c r="G61" s="21" t="n"/>
+      <c r="H61" s="22" t="n"/>
+    </row>
+    <row r="62" ht="16" customHeight="1">
+      <c r="A62" s="9" t="n">
+        <v>2021</v>
+      </c>
+      <c r="B62" s="21" t="n"/>
+      <c r="C62" s="21" t="n"/>
+      <c r="D62" s="21" t="n"/>
+      <c r="E62" s="21" t="n"/>
+      <c r="F62" s="21" t="n"/>
+      <c r="G62" s="21" t="n"/>
+      <c r="H62" s="22" t="n"/>
+    </row>
+    <row r="63" ht="16" customHeight="1">
+      <c r="A63" s="16" t="n">
+        <v>2022</v>
+      </c>
+      <c r="B63" s="21" t="n"/>
+      <c r="C63" s="21" t="n"/>
+      <c r="D63" s="21" t="n"/>
+      <c r="E63" s="21" t="n"/>
+      <c r="F63" s="21" t="n"/>
+      <c r="G63" s="21" t="n"/>
+      <c r="H63" s="22" t="n"/>
+    </row>
+    <row r="64" ht="16" customHeight="1">
+      <c r="A64" s="9" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B64" s="21" t="n"/>
+      <c r="C64" s="21" t="n"/>
+      <c r="D64" s="21" t="n"/>
+      <c r="E64" s="21" t="n"/>
+      <c r="F64" s="21" t="n"/>
+      <c r="G64" s="21" t="n"/>
+      <c r="H64" s="22" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="16" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B65" s="21" t="n"/>
+      <c r="C65" s="21" t="n"/>
+      <c r="D65" s="21" t="n"/>
+      <c r="E65" s="21" t="n"/>
+      <c r="F65" s="21" t="n"/>
+      <c r="G65" s="21" t="n"/>
+      <c r="H65" s="22" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="9" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B66" s="21" t="n"/>
+      <c r="C66" s="21" t="n"/>
+      <c r="D66" s="21" t="n"/>
+      <c r="E66" s="21" t="n"/>
+      <c r="F66" s="21" t="n"/>
+      <c r="G66" s="21" t="n"/>
+      <c r="H66" s="22" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="17" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B67" s="21" t="n"/>
+      <c r="C67" s="21" t="n"/>
+      <c r="D67" s="21" t="n"/>
+      <c r="E67" s="21" t="n"/>
+      <c r="F67" s="21" t="n"/>
+      <c r="G67" s="21" t="n"/>
+      <c r="H67" s="22" t="n"/>
+    </row>
+    <row r="68"/>
+    <row r="69">
+      <c r="A69" s="14" t="inlineStr">
+        <is>
+          <t>Diabetes Selected 4 Drugs</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="15" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="B70" s="21" t="n"/>
+      <c r="C70" s="21" t="n"/>
+      <c r="D70" s="21" t="n"/>
+      <c r="E70" s="21" t="n"/>
+      <c r="F70" s="21" t="n"/>
+      <c r="G70" s="21" t="n"/>
+      <c r="H70" s="22" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="9" t="n">
+        <v>2021</v>
+      </c>
+      <c r="B71" s="21" t="n"/>
+      <c r="C71" s="21" t="n"/>
+      <c r="D71" s="21" t="n"/>
+      <c r="E71" s="21" t="n"/>
+      <c r="F71" s="21" t="n"/>
+      <c r="G71" s="21" t="n"/>
+      <c r="H71" s="22" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="16" t="n">
+        <v>2022</v>
+      </c>
+      <c r="B72" s="21" t="n"/>
+      <c r="C72" s="21" t="n"/>
+      <c r="D72" s="21" t="n"/>
+      <c r="E72" s="21" t="n"/>
+      <c r="F72" s="21" t="n"/>
+      <c r="G72" s="21" t="n"/>
+      <c r="H72" s="22" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="9" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B73" s="21" t="n"/>
+      <c r="C73" s="21" t="n"/>
+      <c r="D73" s="21" t="n"/>
+      <c r="E73" s="21" t="n"/>
+      <c r="F73" s="21" t="n"/>
+      <c r="G73" s="21" t="n"/>
+      <c r="H73" s="22" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="16" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B74" s="21" t="n"/>
+      <c r="C74" s="21" t="n"/>
+      <c r="D74" s="21" t="n"/>
+      <c r="E74" s="21" t="n"/>
+      <c r="F74" s="21" t="n"/>
+      <c r="G74" s="21" t="n"/>
+      <c r="H74" s="22" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="9" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B75" s="21" t="n"/>
+      <c r="C75" s="21" t="n"/>
+      <c r="D75" s="21" t="n"/>
+      <c r="E75" s="21" t="n"/>
+      <c r="F75" s="21" t="n"/>
+      <c r="G75" s="21" t="n"/>
+      <c r="H75" s="22" t="n"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="17" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B76" s="21" t="n"/>
+      <c r="C76" s="21" t="n"/>
+      <c r="D76" s="21" t="n"/>
+      <c r="E76" s="21" t="n"/>
+      <c r="F76" s="21" t="n"/>
+      <c r="G76" s="21" t="n"/>
+      <c r="H76" s="22" t="n"/>
+    </row>
+    <row r="77"/>
+    <row r="78">
+      <c r="A78" s="11" t="inlineStr">
         <is>
           <t>HANConv GNN Performance Analysis</t>
-        </is>
-      </c>
-    </row>
-    <row r="61" ht="16" customHeight="1">
-      <c r="A61" s="13" t="inlineStr">
-        <is>
-          <t>The HANConv GNN achieves lower accuracy (~59-61%) and Macro-F1 (~12-13%) compared to XGBoost (94-95%). This is expected for the following reasons:</t>
-        </is>
-      </c>
-    </row>
-    <row r="62" ht="16" customHeight="1">
-      <c r="A62" s="13" t="inlineStr">
-        <is>
-          <t>1. Class Imbalance: OT (Other Serious) dominates ~60% of the data, while RI (Required Intervention) has only 3-5 samples. The GNN tends to predict the majority class.</t>
-        </is>
-      </c>
-    </row>
-    <row r="63" ht="16" customHeight="1">
-      <c r="A63" s="13" t="inlineStr">
-        <is>
-          <t>2. Graph Structure: With only 15-17 drug nodes and 1,600-1,726 ADR nodes, the heterogeneous graph is relatively sparse for HANConv to learn meaningful attention patterns.</t>
-        </is>
-      </c>
-    </row>
-    <row r="64" ht="16" customHeight="1">
-      <c r="A64" s="13" t="inlineStr">
-        <is>
-          <t>3. Tabular Data Strength: XGBoost and Random Forest excel on structured tabular features with categorical encoding, which is the natural format of FAERS pharmacovigilance data.</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="13" t="inlineStr">
-        <is>
-          <t>4. Data is Complete: The low GNN performance is NOT a data issue. All 20 quarters (2021 Q1 through 2025 Q4) are fully represented in both datasets.</t>
-        </is>
-      </c>
-    </row>
-    <row r="66"/>
-    <row r="67">
-      <c r="A67" s="11" t="inlineStr">
-        <is>
-          <t>Strategies for Improving HANConv GNN Multiclass Performance</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="13" t="inlineStr">
-        <is>
-          <t>To improve multiclass classification accuracy for graph neural networks in future work:</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="13" t="inlineStr">
-        <is>
-          <t>1. Introduce Semantic Node Features: Use pre-trained chemical fingerprint embeddings (e.g., PubChem fingerprints) for drug nodes and biomedical ontology embeddings (e.g., UMLS/MedDRA codes via BioBERT) for reaction (pt_term) nodes instead of degree-based initialization.</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="13" t="inlineStr">
-        <is>
-          <t>2. Class-Balanced Loss Functions: Deploy Class-Weighted Cross-Entropy or Focal Loss to heavily penalize errors on minority classes (e.g., RI, DS) and combat high class imbalance.</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="13" t="inlineStr">
-        <is>
-          <t>3. Homogeneous Knowledge Bridges: Enrich graph topology by incorporating auxiliary homogeneous edges representing drug-drug chemical similarities and reaction-reaction clinical similarities.</t>
-        </is>
-      </c>
-    </row>
-    <row r="72"/>
-    <row r="73">
-      <c r="A73" s="11" t="inlineStr">
-        <is>
-          <t>Scientific Paper Framing (Recommended LaTeX Paragraph)</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" s="13" t="inlineStr">
-        <is>
-          <t>To justify the model choice in your journal manuscript, copy and insert the following paragraph:</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" s="19" t="inlineStr">
-        <is>
-          <t>--------------------------------------------------------------------------------------------------------------------------------------------------------</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" s="20" t="inlineStr">
-        <is>
-          <t>\subsection{Sub-Cohort Analysis and Tabular Model Justification}</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" s="13" t="inlineStr">
-        <is>
-          <t>While the global signal detection pipeline relies on the scale and structural learning capabilities of the heterogeneous</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" s="19" t="inlineStr">
-        <is>
-          <t>HANConv Graph Neural Network (GNN), local sub-cohort analyses---specifically anti-obesity and anti-diabetic cohorts---</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="13" t="inlineStr">
         <is>
-          <t>present distinct structural characteristics. When restricting the reporting network to a narrow subset of anti-obesity agents</t>
+          <t>The HANConv GNN achieves lower accuracy (~59-61%) and Macro-F1 (~12-13%) compared to XGBoost (94-95%). This is expected for the following reasons:</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="13" t="inlineStr">
         <is>
-          <t>(e.g., Semaglutide, Liraglutide, Tirzepatide), the resulting subgraph becomes highly sparse, with a restricted neighborhood</t>
+          <t>1. Class Imbalance: OT (Other Serious) dominates ~60% of the data, while RI (Required Intervention) has only 3-5 samples. The GNN tends to predict the majority class.</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="13" t="inlineStr">
         <is>
-          <t>size that limits the message-passing efficiency of graph attention mechanisms. To overcome this localized sparsity, we deployed</t>
+          <t>2. Graph Structure: With only 15-17 drug nodes and 1,600-1,726 ADR nodes, the heterogeneous graph is relatively sparse for HANConv to learn meaningful attention patterns.</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="13" t="inlineStr">
         <is>
-          <t>tabular gradient-boosted decision trees (XGBoost) alongside the GNN. Empirically, XGBoost demonstrated superior multiclass</t>
+          <t>3. Tabular Data Strength: XGBoost and Random Forest excel on structured tabular features with categorical encoding, which is the natural format of FAERS pharmacovigilance data.</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="13" t="inlineStr">
         <is>
-          <t>outcome prediction accuracy (94.2% to 94.7%) compared to the HANConv GNN (59.6% to 61.2%). Tabular classifiers excel in this</t>
-        </is>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" s="13" t="inlineStr">
-        <is>
-          <t>sub-cohort because the prediction task depends heavily on dense, report-level features (e.g., patient age, weight, administered</t>
-        </is>
-      </c>
-    </row>
+          <t>4. Data is Complete: The low GNN performance is NOT a data issue. All 20 quarters (2021 Q1 through 2025 Q4) are fully represented in both datasets.</t>
+        </is>
+      </c>
+    </row>
+    <row r="84"/>
     <row r="85">
-      <c r="A85" s="13" t="inlineStr">
-        <is>
-          <t>dose, and normalized drug sequence roles) rather than wider topological reporting networks. Consequently, we present XGBoost</t>
+      <c r="A85" s="11" t="inlineStr">
+        <is>
+          <t>Strategies for Improving HANConv GNN Multiclass Performance</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="13" t="inlineStr">
         <is>
-          <t>as the primary predictive engine for the anti-obesity cohort, while maintaining the HANConv GNN architecture for global,</t>
+          <t>To improve multiclass classification accuracy for graph neural networks in future work:</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="13" t="inlineStr">
         <is>
+          <t>1. Introduce Semantic Node Features: Use pre-trained chemical fingerprint embeddings (e.g., PubChem fingerprints) for drug nodes and biomedical ontology embeddings (e.g., UMLS/MedDRA codes via BioBERT) for reaction (pt_term) nodes instead of degree-based initialization.</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="13" t="inlineStr">
+        <is>
+          <t>2. Class-Balanced Loss Functions: Deploy Class-Weighted Cross-Entropy or Focal Loss to heavily penalize errors on minority classes (e.g., RI, DS) and combat high class imbalance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="13" t="inlineStr">
+        <is>
+          <t>3. Homogeneous Knowledge Bridges: Enrich graph topology by incorporating auxiliary homogeneous edges representing drug-drug chemical similarities and reaction-reaction clinical similarities.</t>
+        </is>
+      </c>
+    </row>
+    <row r="90"/>
+    <row r="91">
+      <c r="A91" s="11" t="inlineStr">
+        <is>
+          <t>Scientific Paper Framing (Recommended LaTeX Paragraph)</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="13" t="inlineStr">
+        <is>
+          <t>To justify the model choice in your journal manuscript, copy and insert the following paragraph:</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="19" t="inlineStr">
+        <is>
+          <t>--------------------------------------------------------------------------------------------------------------------------------------------------------</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="20" t="inlineStr">
+        <is>
+          <t>\subsection{Sub-Cohort Analysis and Tabular Model Justification}</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="13" t="inlineStr">
+        <is>
+          <t>While the global signal detection pipeline relies on the scale and structural learning capabilities of the heterogeneous</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="19" t="inlineStr">
+        <is>
+          <t>HANConv Graph Neural Network (GNN), local sub-cohort analyses---specifically anti-obesity and anti-diabetic cohorts---</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="13" t="inlineStr">
+        <is>
+          <t>present distinct structural characteristics. When restricting the reporting network to a narrow subset of anti-obesity agents</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="13" t="inlineStr">
+        <is>
+          <t>(e.g., Semaglutide, Liraglutide, Tirzepatide), the resulting subgraph becomes highly sparse, with a restricted neighborhood</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="13" t="inlineStr">
+        <is>
+          <t>size that limits the message-passing efficiency of graph attention mechanisms. To overcome this localized sparsity, we deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="13" t="inlineStr">
+        <is>
+          <t>tabular gradient-boosted decision trees (XGBoost) alongside the GNN. Empirically, XGBoost demonstrated superior multiclass</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="13" t="inlineStr">
+        <is>
+          <t>outcome prediction accuracy (94.2% to 94.7%) compared to the HANConv GNN (59.6% to 61.2%). Tabular classifiers excel in this</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="13" t="inlineStr">
+        <is>
+          <t>sub-cohort because the prediction task depends heavily on dense, report-level features (e.g., patient age, weight, administered</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="13" t="inlineStr">
+        <is>
+          <t>dose, and normalized drug sequence roles) rather than wider topological reporting networks. Consequently, we present XGBoost</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="13" t="inlineStr">
+        <is>
+          <t>as the primary predictive engine for the anti-obesity cohort, while maintaining the HANConv GNN architecture for global,</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="13" t="inlineStr">
+        <is>
           <t>multi-drug signal detection where network topology is the dominant feature.</t>
         </is>
       </c>
     </row>
-    <row r="88">
-      <c r="A88" s="19" t="inlineStr">
+    <row r="106">
+      <c r="A106" s="19" t="inlineStr">
         <is>
           <t>--------------------------------------------------------------------------------------------------------------------------------------------------------</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="31">
+  <mergeCells count="34">
     <mergeCell ref="A67:H67"/>
     <mergeCell ref="A77:H77"/>
     <mergeCell ref="A24:H24"/>
@@ -1946,6 +2140,7 @@
     <mergeCell ref="A51:H51"/>
     <mergeCell ref="A64:H64"/>
     <mergeCell ref="A82:H82"/>
+    <mergeCell ref="A60:H60"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A79:H79"/>
     <mergeCell ref="A61:H61"/>
@@ -1953,6 +2148,7 @@
     <mergeCell ref="A78:H78"/>
     <mergeCell ref="A69:H69"/>
     <mergeCell ref="A65:H65"/>
+    <mergeCell ref="A66:H66"/>
     <mergeCell ref="A80:H80"/>
     <mergeCell ref="A75:H75"/>
     <mergeCell ref="A74:H74"/>
@@ -1961,6 +2157,7 @@
     <mergeCell ref="A71:H71"/>
     <mergeCell ref="A42:H42"/>
     <mergeCell ref="A76:H76"/>
+    <mergeCell ref="A33:H33"/>
     <mergeCell ref="A23:H23"/>
     <mergeCell ref="A17:H17"/>
     <mergeCell ref="A62:H62"/>
@@ -1968,8 +2165,8 @@
     <mergeCell ref="A81:H81"/>
     <mergeCell ref="A63:H63"/>
     <mergeCell ref="A72:H72"/>
+    <mergeCell ref="A19:H19"/>
     <mergeCell ref="A68:H68"/>
-    <mergeCell ref="A19:H19"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix: Remove duplicate empty Diabetes tables and rebuild all merged ranges from scratch
</commit_message>
<xml_diff>
--- a/dataset/15 Columns Leakage/ML_Multiclass_Model_Comparison_Results.xlsx
+++ b/dataset/15 Columns Leakage/ML_Multiclass_Model_Comparison_Results.xlsx
@@ -612,7 +612,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H106"/>
+  <dimension ref="A1:H87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -1747,394 +1747,203 @@
         <v>342</v>
       </c>
     </row>
-    <row r="59" ht="16" customHeight="1"/>
+    <row r="59" ht="16" customHeight="1">
+      <c r="A59" s="11" t="inlineStr">
+        <is>
+          <t>HANConv GNN Performance Analysis</t>
+        </is>
+      </c>
+    </row>
     <row r="60" ht="16" customHeight="1">
-      <c r="A60" s="14" t="inlineStr">
-        <is>
-          <t>Diabetes All Drugs (10)</t>
+      <c r="A60" s="13" t="inlineStr">
+        <is>
+          <t>The HANConv GNN achieves lower accuracy (~59-61%) and Macro-F1 (~12-13%) compared to XGBoost (94-95%). This is expected for the following reasons:</t>
         </is>
       </c>
     </row>
     <row r="61" ht="16" customHeight="1">
-      <c r="A61" s="15" t="inlineStr">
-        <is>
-          <t>Year</t>
-        </is>
-      </c>
-      <c r="B61" s="21" t="n"/>
-      <c r="C61" s="21" t="n"/>
-      <c r="D61" s="21" t="n"/>
-      <c r="E61" s="21" t="n"/>
-      <c r="F61" s="21" t="n"/>
-      <c r="G61" s="21" t="n"/>
-      <c r="H61" s="22" t="n"/>
+      <c r="A61" s="13" t="inlineStr">
+        <is>
+          <t>1. Class Imbalance: OT (Other Serious) dominates ~60% of the data, while RI (Required Intervention) has only 3-5 samples. The GNN tends to predict the majority class.</t>
+        </is>
+      </c>
     </row>
     <row r="62" ht="16" customHeight="1">
-      <c r="A62" s="9" t="n">
-        <v>2021</v>
-      </c>
-      <c r="B62" s="21" t="n"/>
-      <c r="C62" s="21" t="n"/>
-      <c r="D62" s="21" t="n"/>
-      <c r="E62" s="21" t="n"/>
-      <c r="F62" s="21" t="n"/>
-      <c r="G62" s="21" t="n"/>
-      <c r="H62" s="22" t="n"/>
+      <c r="A62" s="13" t="inlineStr">
+        <is>
+          <t>2. Graph Structure: With only 15-17 drug nodes and 1,600-1,726 ADR nodes, the heterogeneous graph is relatively sparse for HANConv to learn meaningful attention patterns.</t>
+        </is>
+      </c>
     </row>
     <row r="63" ht="16" customHeight="1">
-      <c r="A63" s="16" t="n">
-        <v>2022</v>
-      </c>
-      <c r="B63" s="21" t="n"/>
-      <c r="C63" s="21" t="n"/>
-      <c r="D63" s="21" t="n"/>
-      <c r="E63" s="21" t="n"/>
-      <c r="F63" s="21" t="n"/>
-      <c r="G63" s="21" t="n"/>
-      <c r="H63" s="22" t="n"/>
+      <c r="A63" s="13" t="inlineStr">
+        <is>
+          <t>3. Tabular Data Strength: XGBoost and Random Forest excel on structured tabular features with categorical encoding, which is the natural format of FAERS pharmacovigilance data.</t>
+        </is>
+      </c>
     </row>
     <row r="64" ht="16" customHeight="1">
-      <c r="A64" s="9" t="n">
-        <v>2023</v>
-      </c>
-      <c r="B64" s="21" t="n"/>
-      <c r="C64" s="21" t="n"/>
-      <c r="D64" s="21" t="n"/>
-      <c r="E64" s="21" t="n"/>
-      <c r="F64" s="21" t="n"/>
-      <c r="G64" s="21" t="n"/>
-      <c r="H64" s="22" t="n"/>
-    </row>
-    <row r="65">
-      <c r="A65" s="16" t="n">
-        <v>2024</v>
-      </c>
-      <c r="B65" s="21" t="n"/>
-      <c r="C65" s="21" t="n"/>
-      <c r="D65" s="21" t="n"/>
-      <c r="E65" s="21" t="n"/>
-      <c r="F65" s="21" t="n"/>
-      <c r="G65" s="21" t="n"/>
-      <c r="H65" s="22" t="n"/>
-    </row>
+      <c r="A64" s="13" t="inlineStr">
+        <is>
+          <t>4. Data is Complete: The low GNN performance is NOT a data issue. All 20 quarters (2021 Q1 through 2025 Q4) are fully represented in both datasets.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65"/>
     <row r="66">
-      <c r="A66" s="9" t="n">
-        <v>2025</v>
-      </c>
-      <c r="B66" s="21" t="n"/>
-      <c r="C66" s="21" t="n"/>
-      <c r="D66" s="21" t="n"/>
-      <c r="E66" s="21" t="n"/>
-      <c r="F66" s="21" t="n"/>
-      <c r="G66" s="21" t="n"/>
-      <c r="H66" s="22" t="n"/>
+      <c r="A66" s="11" t="inlineStr">
+        <is>
+          <t>Strategies for Improving HANConv GNN Multiclass Performance</t>
+        </is>
+      </c>
     </row>
     <row r="67">
-      <c r="A67" s="17" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="B67" s="21" t="n"/>
-      <c r="C67" s="21" t="n"/>
-      <c r="D67" s="21" t="n"/>
-      <c r="E67" s="21" t="n"/>
-      <c r="F67" s="21" t="n"/>
-      <c r="G67" s="21" t="n"/>
-      <c r="H67" s="22" t="n"/>
-    </row>
-    <row r="68"/>
+      <c r="A67" s="13" t="inlineStr">
+        <is>
+          <t>To improve multiclass classification accuracy for graph neural networks in future work:</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="13" t="inlineStr">
+        <is>
+          <t>1. Introduce Semantic Node Features: Use pre-trained chemical fingerprint embeddings (e.g., PubChem fingerprints) for drug nodes and biomedical ontology embeddings (e.g., UMLS/MedDRA codes via BioBERT) for reaction (pt_term) nodes instead of degree-based initialization.</t>
+        </is>
+      </c>
+    </row>
     <row r="69">
-      <c r="A69" s="14" t="inlineStr">
-        <is>
-          <t>Diabetes Selected 4 Drugs</t>
+      <c r="A69" s="13" t="inlineStr">
+        <is>
+          <t>2. Class-Balanced Loss Functions: Deploy Class-Weighted Cross-Entropy or Focal Loss to heavily penalize errors on minority classes (e.g., RI, DS) and combat high class imbalance.</t>
         </is>
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="15" t="inlineStr">
-        <is>
-          <t>Year</t>
-        </is>
-      </c>
-      <c r="B70" s="21" t="n"/>
-      <c r="C70" s="21" t="n"/>
-      <c r="D70" s="21" t="n"/>
-      <c r="E70" s="21" t="n"/>
-      <c r="F70" s="21" t="n"/>
-      <c r="G70" s="21" t="n"/>
-      <c r="H70" s="22" t="n"/>
-    </row>
-    <row r="71">
-      <c r="A71" s="9" t="n">
-        <v>2021</v>
-      </c>
-      <c r="B71" s="21" t="n"/>
-      <c r="C71" s="21" t="n"/>
-      <c r="D71" s="21" t="n"/>
-      <c r="E71" s="21" t="n"/>
-      <c r="F71" s="21" t="n"/>
-      <c r="G71" s="21" t="n"/>
-      <c r="H71" s="22" t="n"/>
-    </row>
+      <c r="A70" s="13" t="inlineStr">
+        <is>
+          <t>3. Homogeneous Knowledge Bridges: Enrich graph topology by incorporating auxiliary homogeneous edges representing drug-drug chemical similarities and reaction-reaction clinical similarities.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71"/>
     <row r="72">
-      <c r="A72" s="16" t="n">
-        <v>2022</v>
-      </c>
-      <c r="B72" s="21" t="n"/>
-      <c r="C72" s="21" t="n"/>
-      <c r="D72" s="21" t="n"/>
-      <c r="E72" s="21" t="n"/>
-      <c r="F72" s="21" t="n"/>
-      <c r="G72" s="21" t="n"/>
-      <c r="H72" s="22" t="n"/>
+      <c r="A72" s="11" t="inlineStr">
+        <is>
+          <t>Scientific Paper Framing (Recommended LaTeX Paragraph)</t>
+        </is>
+      </c>
     </row>
     <row r="73">
-      <c r="A73" s="9" t="n">
-        <v>2023</v>
-      </c>
-      <c r="B73" s="21" t="n"/>
-      <c r="C73" s="21" t="n"/>
-      <c r="D73" s="21" t="n"/>
-      <c r="E73" s="21" t="n"/>
-      <c r="F73" s="21" t="n"/>
-      <c r="G73" s="21" t="n"/>
-      <c r="H73" s="22" t="n"/>
+      <c r="A73" s="13" t="inlineStr">
+        <is>
+          <t>To justify the model choice in your journal manuscript, copy and insert the following paragraph:</t>
+        </is>
+      </c>
     </row>
     <row r="74">
-      <c r="A74" s="16" t="n">
-        <v>2024</v>
-      </c>
-      <c r="B74" s="21" t="n"/>
-      <c r="C74" s="21" t="n"/>
-      <c r="D74" s="21" t="n"/>
-      <c r="E74" s="21" t="n"/>
-      <c r="F74" s="21" t="n"/>
-      <c r="G74" s="21" t="n"/>
-      <c r="H74" s="22" t="n"/>
+      <c r="A74" s="19" t="inlineStr">
+        <is>
+          <t>--------------------------------------------------------------------------------------------------------------------------------------------------------</t>
+        </is>
+      </c>
     </row>
     <row r="75">
-      <c r="A75" s="9" t="n">
-        <v>2025</v>
-      </c>
-      <c r="B75" s="21" t="n"/>
-      <c r="C75" s="21" t="n"/>
-      <c r="D75" s="21" t="n"/>
-      <c r="E75" s="21" t="n"/>
-      <c r="F75" s="21" t="n"/>
-      <c r="G75" s="21" t="n"/>
-      <c r="H75" s="22" t="n"/>
+      <c r="A75" s="20" t="inlineStr">
+        <is>
+          <t>\subsection{Sub-Cohort Analysis and Tabular Model Justification}</t>
+        </is>
+      </c>
     </row>
     <row r="76">
-      <c r="A76" s="17" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="B76" s="21" t="n"/>
-      <c r="C76" s="21" t="n"/>
-      <c r="D76" s="21" t="n"/>
-      <c r="E76" s="21" t="n"/>
-      <c r="F76" s="21" t="n"/>
-      <c r="G76" s="21" t="n"/>
-      <c r="H76" s="22" t="n"/>
-    </row>
-    <row r="77"/>
+      <c r="A76" s="13" t="inlineStr">
+        <is>
+          <t>While the global signal detection pipeline relies on the scale and structural learning capabilities of the heterogeneous</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="19" t="inlineStr">
+        <is>
+          <t>HANConv Graph Neural Network (GNN), local sub-cohort analyses---specifically anti-obesity and anti-diabetic cohorts---</t>
+        </is>
+      </c>
+    </row>
     <row r="78">
-      <c r="A78" s="11" t="inlineStr">
-        <is>
-          <t>HANConv GNN Performance Analysis</t>
+      <c r="A78" s="13" t="inlineStr">
+        <is>
+          <t>present distinct structural characteristics. When restricting the reporting network to a narrow subset of anti-obesity agents</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="13" t="inlineStr">
         <is>
-          <t>The HANConv GNN achieves lower accuracy (~59-61%) and Macro-F1 (~12-13%) compared to XGBoost (94-95%). This is expected for the following reasons:</t>
+          <t>(e.g., Semaglutide, Liraglutide, Tirzepatide), the resulting subgraph becomes highly sparse, with a restricted neighborhood</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="13" t="inlineStr">
         <is>
-          <t>1. Class Imbalance: OT (Other Serious) dominates ~60% of the data, while RI (Required Intervention) has only 3-5 samples. The GNN tends to predict the majority class.</t>
+          <t>size that limits the message-passing efficiency of graph attention mechanisms. To overcome this localized sparsity, we deployed</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="13" t="inlineStr">
         <is>
-          <t>2. Graph Structure: With only 15-17 drug nodes and 1,600-1,726 ADR nodes, the heterogeneous graph is relatively sparse for HANConv to learn meaningful attention patterns.</t>
+          <t>tabular gradient-boosted decision trees (XGBoost) alongside the GNN. Empirically, XGBoost demonstrated superior multiclass</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="13" t="inlineStr">
         <is>
-          <t>3. Tabular Data Strength: XGBoost and Random Forest excel on structured tabular features with categorical encoding, which is the natural format of FAERS pharmacovigilance data.</t>
+          <t>outcome prediction accuracy (94.2% to 94.7%) compared to the HANConv GNN (59.6% to 61.2%). Tabular classifiers excel in this</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="13" t="inlineStr">
         <is>
-          <t>4. Data is Complete: The low GNN performance is NOT a data issue. All 20 quarters (2021 Q1 through 2025 Q4) are fully represented in both datasets.</t>
-        </is>
-      </c>
-    </row>
-    <row r="84"/>
+          <t>sub-cohort because the prediction task depends heavily on dense, report-level features (e.g., patient age, weight, administered</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="13" t="inlineStr">
+        <is>
+          <t>dose, and normalized drug sequence roles) rather than wider topological reporting networks. Consequently, we present XGBoost</t>
+        </is>
+      </c>
+    </row>
     <row r="85">
-      <c r="A85" s="11" t="inlineStr">
-        <is>
-          <t>Strategies for Improving HANConv GNN Multiclass Performance</t>
+      <c r="A85" s="13" t="inlineStr">
+        <is>
+          <t>as the primary predictive engine for the anti-obesity cohort, while maintaining the HANConv GNN architecture for global,</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="13" t="inlineStr">
         <is>
-          <t>To improve multiclass classification accuracy for graph neural networks in future work:</t>
+          <t>multi-drug signal detection where network topology is the dominant feature.</t>
         </is>
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="13" t="inlineStr">
-        <is>
-          <t>1. Introduce Semantic Node Features: Use pre-trained chemical fingerprint embeddings (e.g., PubChem fingerprints) for drug nodes and biomedical ontology embeddings (e.g., UMLS/MedDRA codes via BioBERT) for reaction (pt_term) nodes instead of degree-based initialization.</t>
-        </is>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88" s="13" t="inlineStr">
-        <is>
-          <t>2. Class-Balanced Loss Functions: Deploy Class-Weighted Cross-Entropy or Focal Loss to heavily penalize errors on minority classes (e.g., RI, DS) and combat high class imbalance.</t>
-        </is>
-      </c>
-    </row>
-    <row r="89">
-      <c r="A89" s="13" t="inlineStr">
-        <is>
-          <t>3. Homogeneous Knowledge Bridges: Enrich graph topology by incorporating auxiliary homogeneous edges representing drug-drug chemical similarities and reaction-reaction clinical similarities.</t>
-        </is>
-      </c>
-    </row>
-    <row r="90"/>
-    <row r="91">
-      <c r="A91" s="11" t="inlineStr">
-        <is>
-          <t>Scientific Paper Framing (Recommended LaTeX Paragraph)</t>
-        </is>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92" s="13" t="inlineStr">
-        <is>
-          <t>To justify the model choice in your journal manuscript, copy and insert the following paragraph:</t>
-        </is>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" s="19" t="inlineStr">
+      <c r="A87" s="19" t="inlineStr">
         <is>
           <t>--------------------------------------------------------------------------------------------------------------------------------------------------------</t>
         </is>
       </c>
     </row>
-    <row r="94">
-      <c r="A94" s="20" t="inlineStr">
-        <is>
-          <t>\subsection{Sub-Cohort Analysis and Tabular Model Justification}</t>
-        </is>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" s="13" t="inlineStr">
-        <is>
-          <t>While the global signal detection pipeline relies on the scale and structural learning capabilities of the heterogeneous</t>
-        </is>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" s="19" t="inlineStr">
-        <is>
-          <t>HANConv Graph Neural Network (GNN), local sub-cohort analyses---specifically anti-obesity and anti-diabetic cohorts---</t>
-        </is>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" s="13" t="inlineStr">
-        <is>
-          <t>present distinct structural characteristics. When restricting the reporting network to a narrow subset of anti-obesity agents</t>
-        </is>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" s="13" t="inlineStr">
-        <is>
-          <t>(e.g., Semaglutide, Liraglutide, Tirzepatide), the resulting subgraph becomes highly sparse, with a restricted neighborhood</t>
-        </is>
-      </c>
-    </row>
-    <row r="99">
-      <c r="A99" s="13" t="inlineStr">
-        <is>
-          <t>size that limits the message-passing efficiency of graph attention mechanisms. To overcome this localized sparsity, we deployed</t>
-        </is>
-      </c>
-    </row>
-    <row r="100">
-      <c r="A100" s="13" t="inlineStr">
-        <is>
-          <t>tabular gradient-boosted decision trees (XGBoost) alongside the GNN. Empirically, XGBoost demonstrated superior multiclass</t>
-        </is>
-      </c>
-    </row>
-    <row r="101">
-      <c r="A101" s="13" t="inlineStr">
-        <is>
-          <t>outcome prediction accuracy (94.2% to 94.7%) compared to the HANConv GNN (59.6% to 61.2%). Tabular classifiers excel in this</t>
-        </is>
-      </c>
-    </row>
-    <row r="102">
-      <c r="A102" s="13" t="inlineStr">
-        <is>
-          <t>sub-cohort because the prediction task depends heavily on dense, report-level features (e.g., patient age, weight, administered</t>
-        </is>
-      </c>
-    </row>
-    <row r="103">
-      <c r="A103" s="13" t="inlineStr">
-        <is>
-          <t>dose, and normalized drug sequence roles) rather than wider topological reporting networks. Consequently, we present XGBoost</t>
-        </is>
-      </c>
-    </row>
-    <row r="104">
-      <c r="A104" s="13" t="inlineStr">
-        <is>
-          <t>as the primary predictive engine for the anti-obesity cohort, while maintaining the HANConv GNN architecture for global,</t>
-        </is>
-      </c>
-    </row>
-    <row r="105">
-      <c r="A105" s="13" t="inlineStr">
-        <is>
-          <t>multi-drug signal detection where network topology is the dominant feature.</t>
-        </is>
-      </c>
-    </row>
-    <row r="106">
-      <c r="A106" s="19" t="inlineStr">
-        <is>
-          <t>--------------------------------------------------------------------------------------------------------------------------------------------------------</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <mergeCells count="34">
+  <mergeCells count="38">
     <mergeCell ref="A67:H67"/>
     <mergeCell ref="A77:H77"/>
+    <mergeCell ref="A83:H83"/>
+    <mergeCell ref="A59:H59"/>
     <mergeCell ref="A24:H24"/>
     <mergeCell ref="A73:H73"/>
     <mergeCell ref="A51:H51"/>
@@ -2147,14 +1956,16 @@
     <mergeCell ref="A70:H70"/>
     <mergeCell ref="A78:H78"/>
     <mergeCell ref="A69:H69"/>
-    <mergeCell ref="A65:H65"/>
+    <mergeCell ref="A87:H87"/>
     <mergeCell ref="A66:H66"/>
     <mergeCell ref="A80:H80"/>
     <mergeCell ref="A75:H75"/>
+    <mergeCell ref="A84:H84"/>
     <mergeCell ref="A74:H74"/>
     <mergeCell ref="A18:H18"/>
     <mergeCell ref="A21:H21"/>
-    <mergeCell ref="A71:H71"/>
+    <mergeCell ref="A86:H86"/>
+    <mergeCell ref="A85:H85"/>
     <mergeCell ref="A42:H42"/>
     <mergeCell ref="A76:H76"/>
     <mergeCell ref="A33:H33"/>

</xml_diff>

<commit_message>
Update title to mention 15 Columns With Leakage
</commit_message>
<xml_diff>
--- a/dataset/15 Columns Leakage/ML_Multiclass_Model_Comparison_Results.xlsx
+++ b/dataset/15 Columns Leakage/ML_Multiclass_Model_Comparison_Results.xlsx
@@ -628,7 +628,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>FAERS Pediatric Multiclass Outcomes (outc_cod) Prediction Comparison</t>
+          <t>FAERS Pediatric Multiclass Outcomes (outc_cod) Prediction Comparison — 15 Columns (With Leakage)</t>
         </is>
       </c>
     </row>
@@ -1789,7 +1789,6 @@
         </is>
       </c>
     </row>
-    <row r="65"/>
     <row r="66">
       <c r="A66" s="11" t="inlineStr">
         <is>
@@ -1825,7 +1824,6 @@
         </is>
       </c>
     </row>
-    <row r="71"/>
     <row r="72">
       <c r="A72" s="11" t="inlineStr">
         <is>

</xml_diff>